<commit_message>
Recheck POI icon positions and shrink markers
</commit_message>
<xml_diff>
--- a/map-data/baoshan-poi-coordinates-v1.9.6.xlsx
+++ b/map-data/baoshan-poi-coordinates-v1.9.6.xlsx
@@ -9,13 +9,11 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="宝山POI坐标" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="图例与规则" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="宝山路网坐标" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="坐标说明" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="坐标说明" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'宝山POI坐标'!$A$1:$L$41</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'图例与规则'!$A$1:$D$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'宝山路网坐标'!$A$1:$E$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'宝山POI坐标'!$A$1:$N$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'图例与规则'!$A$1:$D$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -433,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L41"/>
+  <dimension ref="A1:N41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -442,12 +440,14 @@
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="45" customWidth="1" min="10" max="10"/>
-    <col width="48" customWidth="1" min="11" max="11"/>
-    <col width="32" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="45" customWidth="1" min="12" max="12"/>
+    <col width="48" customWidth="1" min="13" max="13"/>
+    <col width="32" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -468,45 +468,55 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>地图X</t>
+          <t>路网X</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>地图Y</t>
+          <t>路网Y</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>图标X</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>图标Y</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>坐标版本</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>垃圾点类型</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>通行限制</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>用户端显示</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>作用用途</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>找路说明</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>数据来源</t>
         </is>
@@ -535,26 +545,32 @@
         <v>141</v>
       </c>
       <c r="F2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
+        <v>352</v>
+      </c>
+      <c r="G2" t="n">
+        <v>141</v>
+      </c>
+      <c r="H2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
         <is>
           <t>医务室，具体服务以校内公告为准。</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>北入口西侧、北部绿地旁。</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>用户提供的校园平面图</t>
         </is>
@@ -583,26 +599,32 @@
         <v>220</v>
       </c>
       <c r="F3" t="n">
-        <v>2</v>
-      </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
+        <v>193</v>
+      </c>
+      <c r="G3" t="n">
+        <v>220</v>
+      </c>
+      <c r="H3" t="n">
+        <v>3</v>
+      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
         <is>
           <t>教工集体宿舍，具体服务以校内公告为准。</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>位置依据用户提供的校园平面图；门牌及当前通行条件待确认。</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>用户提供的校园平面图</t>
         </is>
@@ -631,26 +653,32 @@
         <v>270</v>
       </c>
       <c r="F4" t="n">
-        <v>2</v>
-      </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
+        <v>216</v>
+      </c>
+      <c r="G4" t="n">
+        <v>318</v>
+      </c>
+      <c r="H4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
         <is>
           <t>建工系综合实训楼，具体服务以校内公告为准。</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>位置依据用户提供的校园平面图；门牌及当前通行条件待确认。</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>用户提供的校园平面图</t>
         </is>
@@ -679,26 +707,32 @@
         <v>341</v>
       </c>
       <c r="F5" t="n">
-        <v>2</v>
-      </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
+        <v>174</v>
+      </c>
+      <c r="G5" t="n">
+        <v>369</v>
+      </c>
+      <c r="H5" t="n">
+        <v>3</v>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
         <is>
           <t>实训中心楼，具体服务以校内公告为准。</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>位置依据用户提供的校园平面图；门牌及当前通行条件待确认。</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>用户提供的校园平面图</t>
         </is>
@@ -727,26 +761,32 @@
         <v>333</v>
       </c>
       <c r="F6" t="n">
-        <v>2</v>
-      </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
+        <v>466</v>
+      </c>
+      <c r="G6" t="n">
+        <v>368</v>
+      </c>
+      <c r="H6" t="n">
+        <v>3</v>
+      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
         <is>
           <t>教学大楼，具体服务以校内公告为准。</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>位置依据用户提供的校园平面图；门牌及当前通行条件待确认。</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>用户提供的校园平面图</t>
         </is>
@@ -775,26 +815,32 @@
         <v>195</v>
       </c>
       <c r="F7" t="n">
-        <v>2</v>
-      </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
+        <v>571</v>
+      </c>
+      <c r="G7" t="n">
+        <v>195</v>
+      </c>
+      <c r="H7" t="n">
+        <v>3</v>
+      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
         <is>
           <t>学生活动中心，具体服务以校内公告为准。</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>位置依据用户提供的校园平面图；门牌及当前通行条件待确认。</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>用户提供的校园平面图</t>
         </is>
@@ -823,26 +869,32 @@
         <v>240</v>
       </c>
       <c r="F8" t="n">
-        <v>2</v>
-      </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
+        <v>545</v>
+      </c>
+      <c r="G8" t="n">
+        <v>240</v>
+      </c>
+      <c r="H8" t="n">
+        <v>3</v>
+      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
         <is>
           <t>圆形会议室，具体服务以校内公告为准。</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>位置依据用户提供的校园平面图；门牌及当前通行条件待确认。</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>用户提供的校园平面图</t>
         </is>
@@ -871,26 +923,32 @@
         <v>262</v>
       </c>
       <c r="F9" t="n">
-        <v>2</v>
-      </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
+        <v>610</v>
+      </c>
+      <c r="G9" t="n">
+        <v>262</v>
+      </c>
+      <c r="H9" t="n">
+        <v>3</v>
+      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
         <is>
           <t>阶梯教室，具体服务以校内公告为准。</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>位置依据用户提供的校园平面图；门牌及当前通行条件待确认。</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>用户提供的校园平面图</t>
         </is>
@@ -919,26 +977,32 @@
         <v>439</v>
       </c>
       <c r="F10" t="n">
-        <v>2</v>
-      </c>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
+        <v>345</v>
+      </c>
+      <c r="G10" t="n">
+        <v>439</v>
+      </c>
+      <c r="H10" t="n">
+        <v>3</v>
+      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
         <is>
           <t>图文信息楼，具体服务以校内公告为准。</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>位置依据用户提供的校园平面图；门牌及当前通行条件待确认。</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>用户提供的校园平面图</t>
         </is>
@@ -967,26 +1031,32 @@
         <v>480</v>
       </c>
       <c r="F11" t="n">
-        <v>2</v>
-      </c>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
+        <v>591</v>
+      </c>
+      <c r="G11" t="n">
+        <v>480</v>
+      </c>
+      <c r="H11" t="n">
+        <v>3</v>
+      </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
         <is>
           <t>办公楼，具体服务以校内公告为准。</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>位置依据用户提供的校园平面图；门牌及当前通行条件待确认。</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t>用户提供的校园平面图</t>
         </is>
@@ -1015,26 +1085,32 @@
         <v>421</v>
       </c>
       <c r="F12" t="n">
-        <v>2</v>
-      </c>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
+        <v>572</v>
+      </c>
+      <c r="G12" t="n">
+        <v>421</v>
+      </c>
+      <c r="H12" t="n">
+        <v>3</v>
+      </c>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
         <is>
           <t>报告厅，具体服务以校内公告为准。</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="M12" t="inlineStr">
         <is>
           <t>位置依据用户提供的校园平面图；门牌及当前通行条件待确认。</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
+      <c r="N12" t="inlineStr">
         <is>
           <t>用户提供的校园平面图</t>
         </is>
@@ -1063,26 +1139,32 @@
         <v>175</v>
       </c>
       <c r="F13" t="n">
-        <v>2</v>
-      </c>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
+        <v>731</v>
+      </c>
+      <c r="G13" t="n">
+        <v>175</v>
+      </c>
+      <c r="H13" t="n">
+        <v>3</v>
+      </c>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
         <is>
           <t>用于室内体育锻炼和体育活动。具体运动项目、开放时段及预约要求以场馆通知为准。</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="M13" t="inlineStr">
         <is>
           <t>位置依据用户提供的校园平面图；门牌及当前通行条件待确认。</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="N13" t="inlineStr">
         <is>
           <t>用户提供的校园平面图</t>
         </is>
@@ -1111,26 +1193,32 @@
         <v>285</v>
       </c>
       <c r="F14" t="n">
-        <v>2</v>
-      </c>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
+        <v>718</v>
+      </c>
+      <c r="G14" t="n">
+        <v>285</v>
+      </c>
+      <c r="H14" t="n">
+        <v>3</v>
+      </c>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
         <is>
           <t>用于体育教学、集体训练和日常体育活动。雨天使用及场地安排以校内通知为准。</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="M14" t="inlineStr">
         <is>
           <t>位置依据用户提供的校园平面图；门牌及当前通行条件待确认。</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
+      <c r="N14" t="inlineStr">
         <is>
           <t>用户提供的校园平面图</t>
         </is>
@@ -1159,26 +1247,32 @@
         <v>379</v>
       </c>
       <c r="F15" t="n">
-        <v>2</v>
-      </c>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
+        <v>714</v>
+      </c>
+      <c r="G15" t="n">
+        <v>379</v>
+      </c>
+      <c r="H15" t="n">
+        <v>3</v>
+      </c>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
         <is>
           <t>用于打球、球类练习和日常体育锻炼。具体球类项目、场地使用规则及预约要求以现场标识和校内通知为准。</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="M15" t="inlineStr">
         <is>
           <t>位置依据用户提供的校园平面图；门牌及当前通行条件待确认。</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
+      <c r="N15" t="inlineStr">
         <is>
           <t>用户提供的校园平面图</t>
         </is>
@@ -1207,26 +1301,32 @@
         <v>352</v>
       </c>
       <c r="F16" t="n">
-        <v>2</v>
-      </c>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
+        <v>884</v>
+      </c>
+      <c r="G16" t="n">
+        <v>352</v>
+      </c>
+      <c r="H16" t="n">
+        <v>3</v>
+      </c>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
         <is>
           <t>用于跑步、田径练习和日常体育锻炼。足球等场内活动及场地使用安排以校内通知为准。</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
+      <c r="M16" t="inlineStr">
         <is>
           <t>位置依据用户提供的校园平面图；门牌及当前通行条件待确认。</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr">
+      <c r="N16" t="inlineStr">
         <is>
           <t>用户提供的校园平面图</t>
         </is>
@@ -1255,26 +1355,32 @@
         <v>540</v>
       </c>
       <c r="F17" t="n">
-        <v>2</v>
-      </c>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
+        <v>751</v>
+      </c>
+      <c r="G17" t="n">
+        <v>540</v>
+      </c>
+      <c r="H17" t="n">
+        <v>3</v>
+      </c>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
         <is>
           <t>男生宿舍，具体服务以校内公告为准。</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
+      <c r="M17" t="inlineStr">
         <is>
           <t>位置依据用户提供的校园平面图；门牌及当前通行条件待确认。</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr">
+      <c r="N17" t="inlineStr">
         <is>
           <t>用户提供的校园平面图</t>
         </is>
@@ -1303,26 +1409,32 @@
         <v>543</v>
       </c>
       <c r="F18" t="n">
-        <v>2</v>
-      </c>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
+        <v>895</v>
+      </c>
+      <c r="G18" t="n">
+        <v>543</v>
+      </c>
+      <c r="H18" t="n">
+        <v>3</v>
+      </c>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
         <is>
           <t>女生宿舍，具体服务以校内公告为准。</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
+      <c r="M18" t="inlineStr">
         <is>
           <t>位置依据用户提供的校园平面图；门牌及当前通行条件待确认。</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr">
+      <c r="N18" t="inlineStr">
         <is>
           <t>用户提供的校园平面图</t>
         </is>
@@ -1351,26 +1463,32 @@
         <v>582</v>
       </c>
       <c r="F19" t="n">
-        <v>2</v>
-      </c>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
+        <v>753</v>
+      </c>
+      <c r="G19" t="n">
+        <v>582</v>
+      </c>
+      <c r="H19" t="n">
+        <v>3</v>
+      </c>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
         <is>
           <t>食堂，具体服务以校内公告为准。</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
+      <c r="M19" t="inlineStr">
         <is>
           <t>位置依据用户提供的校园平面图；门牌及当前通行条件待确认。</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr">
+      <c r="N19" t="inlineStr">
         <is>
           <t>用户提供的校园平面图</t>
         </is>
@@ -1399,26 +1517,32 @@
         <v>583</v>
       </c>
       <c r="F20" t="n">
-        <v>2</v>
-      </c>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
+        <v>894</v>
+      </c>
+      <c r="G20" t="n">
+        <v>583</v>
+      </c>
+      <c r="H20" t="n">
+        <v>3</v>
+      </c>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
         <is>
           <t>浴室，具体服务以校内公告为准。</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr">
+      <c r="M20" t="inlineStr">
         <is>
           <t>位置依据用户提供的校园平面图；门牌及当前通行条件待确认。</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr">
+      <c r="N20" t="inlineStr">
         <is>
           <t>用户提供的校园平面图</t>
         </is>
@@ -1447,26 +1571,32 @@
         <v>424</v>
       </c>
       <c r="F21" t="n">
-        <v>2</v>
-      </c>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr">
+        <v>87</v>
+      </c>
+      <c r="G21" t="n">
+        <v>424</v>
+      </c>
+      <c r="H21" t="n">
+        <v>3</v>
+      </c>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="L21" t="inlineStr">
         <is>
           <t>建筑实践园，具体服务以校内公告为准。</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
+      <c r="M21" t="inlineStr">
         <is>
           <t>位置依据用户提供的校园平面图；门牌及当前通行条件待确认。</t>
         </is>
       </c>
-      <c r="L21" t="inlineStr">
+      <c r="N21" t="inlineStr">
         <is>
           <t>用户提供的校园平面图</t>
         </is>
@@ -1495,26 +1625,32 @@
         <v>427</v>
       </c>
       <c r="F22" t="n">
-        <v>2</v>
-      </c>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr">
+        <v>174</v>
+      </c>
+      <c r="G22" t="n">
+        <v>427</v>
+      </c>
+      <c r="H22" t="n">
+        <v>3</v>
+      </c>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="L22" t="inlineStr">
         <is>
           <t>土木工程实践园，具体服务以校内公告为准。</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr">
+      <c r="M22" t="inlineStr">
         <is>
           <t>位置依据用户提供的校园平面图；门牌及当前通行条件待确认。</t>
         </is>
       </c>
-      <c r="L22" t="inlineStr">
+      <c r="N22" t="inlineStr">
         <is>
           <t>用户提供的校园平面图</t>
         </is>
@@ -1543,26 +1679,32 @@
         <v>466</v>
       </c>
       <c r="F23" t="n">
-        <v>2</v>
-      </c>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr">
+        <v>215</v>
+      </c>
+      <c r="G23" t="n">
+        <v>466</v>
+      </c>
+      <c r="H23" t="n">
+        <v>3</v>
+      </c>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
+      <c r="L23" t="inlineStr">
         <is>
           <t>绿色建筑创新中心，具体服务以校内公告为准。</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr">
+      <c r="M23" t="inlineStr">
         <is>
           <t>位置依据用户提供的校园平面图；门牌及当前通行条件待确认。</t>
         </is>
       </c>
-      <c r="L23" t="inlineStr">
+      <c r="N23" t="inlineStr">
         <is>
           <t>用户提供的校园平面图</t>
         </is>
@@ -1591,26 +1733,32 @@
         <v>492</v>
       </c>
       <c r="F24" t="n">
-        <v>2</v>
-      </c>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr">
+        <v>153</v>
+      </c>
+      <c r="G24" t="n">
+        <v>492</v>
+      </c>
+      <c r="H24" t="n">
+        <v>3</v>
+      </c>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
+      <c r="L24" t="inlineStr">
         <is>
           <t>园林校内实践园，具体服务以校内公告为准。</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr">
+      <c r="M24" t="inlineStr">
         <is>
           <t>位置依据用户提供的校园平面图；门牌及当前通行条件待确认。</t>
         </is>
       </c>
-      <c r="L24" t="inlineStr">
+      <c r="N24" t="inlineStr">
         <is>
           <t>用户提供的校园平面图</t>
         </is>
@@ -1639,26 +1787,32 @@
         <v>564</v>
       </c>
       <c r="F25" t="n">
-        <v>2</v>
-      </c>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr">
+        <v>215</v>
+      </c>
+      <c r="G25" t="n">
+        <v>564</v>
+      </c>
+      <c r="H25" t="n">
+        <v>3</v>
+      </c>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr">
+      <c r="L25" t="inlineStr">
         <is>
           <t>建筑自然环境设计与控制实训室，具体服务以校内公告为准。</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr">
+      <c r="M25" t="inlineStr">
         <is>
           <t>位置依据用户提供的校园平面图；门牌及当前通行条件待确认。</t>
         </is>
       </c>
-      <c r="L25" t="inlineStr">
+      <c r="N25" t="inlineStr">
         <is>
           <t>用户提供的校园平面图</t>
         </is>
@@ -1687,26 +1841,32 @@
         <v>244</v>
       </c>
       <c r="F26" t="n">
-        <v>2</v>
-      </c>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr">
+        <v>276</v>
+      </c>
+      <c r="G26" t="n">
+        <v>244</v>
+      </c>
+      <c r="H26" t="n">
+        <v>3</v>
+      </c>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
         <is>
           <t>水泵房，具体服务以校内公告为准。</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr">
+      <c r="M26" t="inlineStr">
         <is>
           <t>位置依据用户提供的校园平面图；门牌及当前通行条件待确认。</t>
         </is>
       </c>
-      <c r="L26" t="inlineStr">
+      <c r="N26" t="inlineStr">
         <is>
           <t>用户提供的校园平面图</t>
         </is>
@@ -1735,26 +1895,32 @@
         <v>275</v>
       </c>
       <c r="F27" t="n">
-        <v>2</v>
-      </c>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
+        <v>286</v>
+      </c>
+      <c r="G27" t="n">
+        <v>275</v>
+      </c>
+      <c r="H27" t="n">
+        <v>3</v>
+      </c>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
         <is>
           <t>配电所，具体服务以校内公告为准。</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr">
+      <c r="M27" t="inlineStr">
         <is>
           <t>位置依据用户提供的校园平面图；门牌及当前通行条件待确认。</t>
         </is>
       </c>
-      <c r="L27" t="inlineStr">
+      <c r="N27" t="inlineStr">
         <is>
           <t>用户提供的校园平面图</t>
         </is>
@@ -1783,26 +1949,32 @@
         <v>99</v>
       </c>
       <c r="F28" t="n">
-        <v>2</v>
-      </c>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr">
+        <v>466</v>
+      </c>
+      <c r="G28" t="n">
+        <v>107</v>
+      </c>
+      <c r="H28" t="n">
+        <v>3</v>
+      </c>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
         <is>
           <t>北入口，具体服务以校内公告为准。</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr">
+      <c r="M28" t="inlineStr">
         <is>
           <t>位置依据用户提供的校园平面图；门牌及当前通行条件待确认。</t>
         </is>
       </c>
-      <c r="L28" t="inlineStr">
+      <c r="N28" t="inlineStr">
         <is>
           <t>用户提供的校园平面图</t>
         </is>
@@ -1831,26 +2003,32 @@
         <v>627</v>
       </c>
       <c r="F29" t="n">
-        <v>2</v>
-      </c>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J29" t="inlineStr">
+        <v>469</v>
+      </c>
+      <c r="G29" t="n">
+        <v>620</v>
+      </c>
+      <c r="H29" t="n">
+        <v>3</v>
+      </c>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
         <is>
           <t>南入口，具体服务以校内公告为准。</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr">
+      <c r="M29" t="inlineStr">
         <is>
           <t>位置依据用户提供的校园平面图；门牌及当前通行条件待确认。</t>
         </is>
       </c>
-      <c r="L29" t="inlineStr">
+      <c r="N29" t="inlineStr">
         <is>
           <t>用户提供的校园平面图</t>
         </is>
@@ -1879,26 +2057,32 @@
         <v>275</v>
       </c>
       <c r="F30" t="n">
-        <v>2</v>
-      </c>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J30" t="inlineStr">
+        <v>468</v>
+      </c>
+      <c r="G30" t="n">
+        <v>275</v>
+      </c>
+      <c r="H30" t="n">
+        <v>3</v>
+      </c>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
         <is>
           <t>校园景观大道，具体服务以校内公告为准。</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr">
+      <c r="M30" t="inlineStr">
         <is>
           <t>位置依据用户提供的校园平面图；门牌及当前通行条件待确认。</t>
         </is>
       </c>
-      <c r="L30" t="inlineStr">
+      <c r="N30" t="inlineStr">
         <is>
           <t>用户提供的校园平面图</t>
         </is>
@@ -1927,26 +2111,32 @@
         <v>100</v>
       </c>
       <c r="F31" t="n">
-        <v>2</v>
-      </c>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J31" t="inlineStr">
+        <v>589</v>
+      </c>
+      <c r="G31" t="n">
+        <v>100</v>
+      </c>
+      <c r="H31" t="n">
+        <v>3</v>
+      </c>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
         <is>
           <t>杨鑫路公交站点，具体服务以校内公告为准。</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr">
+      <c r="M31" t="inlineStr">
         <is>
           <t>位置依据用户提供的校园平面图；门牌及当前通行条件待确认。</t>
         </is>
       </c>
-      <c r="L31" t="inlineStr">
+      <c r="N31" t="inlineStr">
         <is>
           <t>用户提供的校园平面图</t>
         </is>
@@ -1975,26 +2165,32 @@
         <v>463</v>
       </c>
       <c r="F32" t="n">
-        <v>2</v>
-      </c>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J32" t="inlineStr">
+        <v>987</v>
+      </c>
+      <c r="G32" t="n">
+        <v>463</v>
+      </c>
+      <c r="H32" t="n">
+        <v>3</v>
+      </c>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
         <is>
           <t>梅林路公交站点，具体服务以校内公告为准。</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr">
+      <c r="M32" t="inlineStr">
         <is>
           <t>位置依据用户提供的校园平面图；门牌及当前通行条件待确认。</t>
         </is>
       </c>
-      <c r="L32" t="inlineStr">
+      <c r="N32" t="inlineStr">
         <is>
           <t>用户提供的校园平面图</t>
         </is>
@@ -2023,30 +2219,36 @@
         <v>397</v>
       </c>
       <c r="F33" t="n">
-        <v>2</v>
-      </c>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr">
+        <v>692</v>
+      </c>
+      <c r="G33" t="n">
+        <v>393</v>
+      </c>
+      <c r="H33" t="n">
+        <v>3</v>
+      </c>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr">
         <is>
           <t>event-only</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr">
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
         <is>
           <t>连接球场西侧的校园出入口；通常关闭，仅在举办活动时开放。</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr">
+      <c r="M33" t="inlineStr">
         <is>
           <t>位于风雨操场下方、球场左侧；请先确认现场是否开放。</t>
         </is>
       </c>
-      <c r="L33" t="inlineStr">
+      <c r="N33" t="inlineStr">
         <is>
           <t>用户提供的校园平面图</t>
         </is>
@@ -2075,30 +2277,36 @@
         <v>169</v>
       </c>
       <c r="F34" t="n">
-        <v>2</v>
-      </c>
-      <c r="G34" t="inlineStr">
+        <v>224</v>
+      </c>
+      <c r="G34" t="n">
+        <v>169</v>
+      </c>
+      <c r="H34" t="n">
+        <v>3</v>
+      </c>
+      <c r="I34" t="inlineStr">
         <is>
           <t>station</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J34" t="inlineStr">
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
         <is>
           <t>集中投放生活垃圾的垃圾站。请按校内分类要求投放。</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr">
+      <c r="M34" t="inlineStr">
         <is>
           <t>位于校区西北侧道路旁；具体开放和分类要求以现场标识为准。</t>
         </is>
       </c>
-      <c r="L34" t="inlineStr">
+      <c r="N34" t="inlineStr">
         <is>
           <t>用户提供的校园平面图图例</t>
         </is>
@@ -2127,30 +2335,36 @@
         <v>524</v>
       </c>
       <c r="F35" t="n">
-        <v>2</v>
-      </c>
-      <c r="G35" t="inlineStr">
+        <v>922</v>
+      </c>
+      <c r="G35" t="n">
+        <v>526</v>
+      </c>
+      <c r="H35" t="n">
+        <v>3</v>
+      </c>
+      <c r="I35" t="inlineStr">
         <is>
           <t>station</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J35" t="inlineStr">
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
         <is>
           <t>集中投放生活垃圾的垃圾站。请按校内分类要求投放。</t>
         </is>
       </c>
-      <c r="K35" t="inlineStr">
+      <c r="M35" t="inlineStr">
         <is>
           <t>位于校区东南侧道路旁；具体开放和分类要求以现场标识为准。</t>
         </is>
       </c>
-      <c r="L35" t="inlineStr">
+      <c r="N35" t="inlineStr">
         <is>
           <t>用户提供的校园平面图图例</t>
         </is>
@@ -2179,30 +2393,36 @@
         <v>213</v>
       </c>
       <c r="F36" t="n">
-        <v>2</v>
-      </c>
-      <c r="G36" t="inlineStr">
+        <v>676</v>
+      </c>
+      <c r="G36" t="n">
+        <v>213</v>
+      </c>
+      <c r="H36" t="n">
+        <v>3</v>
+      </c>
+      <c r="I36" t="inlineStr">
         <is>
           <t>bin</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J36" t="inlineStr">
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
         <is>
           <t>可投放少量日常垃圾的垃圾桶，请按现场分类标识投放。</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr">
+      <c r="M36" t="inlineStr">
         <is>
           <t>位于校园道路或运动场周边；请以现场位置和分类标识为准。</t>
         </is>
       </c>
-      <c r="L36" t="inlineStr">
+      <c r="N36" t="inlineStr">
         <is>
           <t>用户提供的校园平面图图例</t>
         </is>
@@ -2231,30 +2451,36 @@
         <v>241</v>
       </c>
       <c r="F37" t="n">
-        <v>2</v>
-      </c>
-      <c r="G37" t="inlineStr">
+        <v>676</v>
+      </c>
+      <c r="G37" t="n">
+        <v>241</v>
+      </c>
+      <c r="H37" t="n">
+        <v>3</v>
+      </c>
+      <c r="I37" t="inlineStr">
         <is>
           <t>bin</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J37" t="inlineStr">
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
         <is>
           <t>可投放少量日常垃圾的垃圾桶，请按现场分类标识投放。</t>
         </is>
       </c>
-      <c r="K37" t="inlineStr">
+      <c r="M37" t="inlineStr">
         <is>
           <t>位于校园道路或运动场周边；请以现场位置和分类标识为准。</t>
         </is>
       </c>
-      <c r="L37" t="inlineStr">
+      <c r="N37" t="inlineStr">
         <is>
           <t>用户提供的校园平面图图例</t>
         </is>
@@ -2283,30 +2509,36 @@
         <v>271</v>
       </c>
       <c r="F38" t="n">
-        <v>2</v>
-      </c>
-      <c r="G38" t="inlineStr">
+        <v>676</v>
+      </c>
+      <c r="G38" t="n">
+        <v>271</v>
+      </c>
+      <c r="H38" t="n">
+        <v>3</v>
+      </c>
+      <c r="I38" t="inlineStr">
         <is>
           <t>bin</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J38" t="inlineStr">
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
         <is>
           <t>可投放少量日常垃圾的垃圾桶，请按现场分类标识投放。</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr">
+      <c r="M38" t="inlineStr">
         <is>
           <t>位于校园道路或运动场周边；请以现场位置和分类标识为准。</t>
         </is>
       </c>
-      <c r="L38" t="inlineStr">
+      <c r="N38" t="inlineStr">
         <is>
           <t>用户提供的校园平面图图例</t>
         </is>
@@ -2335,30 +2567,36 @@
         <v>329</v>
       </c>
       <c r="F39" t="n">
-        <v>2</v>
-      </c>
-      <c r="G39" t="inlineStr">
+        <v>675</v>
+      </c>
+      <c r="G39" t="n">
+        <v>329</v>
+      </c>
+      <c r="H39" t="n">
+        <v>3</v>
+      </c>
+      <c r="I39" t="inlineStr">
         <is>
           <t>bin</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J39" t="inlineStr">
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
         <is>
           <t>可投放少量日常垃圾的垃圾桶，请按现场分类标识投放。</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr">
+      <c r="M39" t="inlineStr">
         <is>
           <t>位于校园道路或运动场周边；请以现场位置和分类标识为准。</t>
         </is>
       </c>
-      <c r="L39" t="inlineStr">
+      <c r="N39" t="inlineStr">
         <is>
           <t>用户提供的校园平面图图例</t>
         </is>
@@ -2387,30 +2625,36 @@
         <v>330</v>
       </c>
       <c r="F40" t="n">
-        <v>2</v>
-      </c>
-      <c r="G40" t="inlineStr">
+        <v>745</v>
+      </c>
+      <c r="G40" t="n">
+        <v>330</v>
+      </c>
+      <c r="H40" t="n">
+        <v>3</v>
+      </c>
+      <c r="I40" t="inlineStr">
         <is>
           <t>bin</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J40" t="inlineStr">
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
         <is>
           <t>可投放少量日常垃圾的垃圾桶，请按现场分类标识投放。</t>
         </is>
       </c>
-      <c r="K40" t="inlineStr">
+      <c r="M40" t="inlineStr">
         <is>
           <t>位于校园道路或运动场周边；请以现场位置和分类标识为准。</t>
         </is>
       </c>
-      <c r="L40" t="inlineStr">
+      <c r="N40" t="inlineStr">
         <is>
           <t>用户提供的校园平面图图例</t>
         </is>
@@ -2439,37 +2683,43 @@
         <v>495</v>
       </c>
       <c r="F41" t="n">
-        <v>2</v>
-      </c>
-      <c r="G41" t="inlineStr">
+        <v>669</v>
+      </c>
+      <c r="G41" t="n">
+        <v>495</v>
+      </c>
+      <c r="H41" t="n">
+        <v>3</v>
+      </c>
+      <c r="I41" t="inlineStr">
         <is>
           <t>bin</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J41" t="inlineStr">
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
         <is>
           <t>可投放少量日常垃圾的垃圾桶，请按现场分类标识投放。</t>
         </is>
       </c>
-      <c r="K41" t="inlineStr">
+      <c r="M41" t="inlineStr">
         <is>
           <t>位于校园道路或运动场周边；请以现场位置和分类标识为准。</t>
         </is>
       </c>
-      <c r="L41" t="inlineStr">
+      <c r="N41" t="inlineStr">
         <is>
           <t>用户提供的校园平面图图例</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L41"/>
+  <autoFilter ref="A1:N41"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2480,13 +2730,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="65" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2502,7 +2752,7 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>导航/交互规则</t>
+          <t>本次核对结果</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
@@ -2524,51 +2774,51 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>作为宝山校区地图背景；不显示红/蓝/橙/紫施工标线</t>
+          <t>保持不变</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>清理后的用户底图</t>
+          <t>用户提供底图清理版</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>红线障碍</t>
+          <t>建筑圆点</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>不显示</t>
+          <t>缩小圆点 + 亮眼浅蓝说明</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>作为不可穿越边界，过滤连接边；蓝色建筑内部通路保留</t>
+          <t>图标坐标存于 markerX/markerY；路网坐标 mapX/mapY 保持不变</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>用户标注图</t>
+          <t>本次入口复核</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>蓝线一层道路</t>
+          <t>垃圾站/垃圾桶</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>不显示</t>
+          <t>黄色圆点 + 亮眼浅蓝说明</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>1 层步行边；建筑内部蓝线按普通学生日常可通行处理</t>
+          <t>8 个黄点逐一复核；右下垃圾站对齐东南边界黄点</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -2580,17 +2830,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>橙线二层道路</t>
+          <t>未探索区域</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>不显示</t>
+          <t>灰色遮罩</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2 层步行边；与蓝线相交不自动换层</t>
+          <t>显示范围使用 displayPoints；路网排除范围不变，区域内 POI 不显示</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -2602,115 +2852,27 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>紫线楼梯</t>
+          <t>路网与导航</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>不显示</t>
+          <t>常规不显示，导航显示箭头</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>全图唯一垂直交通连接，普通步行可用；避开楼梯模式过滤</t>
+          <t>保持不变</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>用户澄清</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>黄色大点垃圾站</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>黄色圆点 + 说明</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>可点击查看垃圾站用途</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>用户标注图</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>黄色小点垃圾桶</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>黄色圆点 + 说明</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>可点击查看垃圾桶用途</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>用户标注图</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>黑色斜杠区域</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>灰色遮罩</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>不显示区域内 POI；不可点击、不可规划</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>用户标注图</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>活动出入口</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>橙色圆点</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>球场左侧大型出入口通常关闭，仅活动时开放</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>用户澄清</t>
+          <t>上一任务</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D10"/>
+  <autoFilter ref="A1:D6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2721,497 +2883,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="90" customWidth="1" min="4" max="4"/>
-    <col width="44" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>类型</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>编号</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>楼层</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>坐标点（X,Y）</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>说明</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>通路</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>north-west</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>470,96; 470,129; 410,129; 350,129; 300,144; 250,167; 220,208; 210,265; 210,335; 250,369; 330,369; 400,369; 470,369</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>仅作为导航记忆数据，常规地图不绘制</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>通路</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>north-east</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>470,96; 470,129; 560,129; 650,129; 720,133; 820,138; 900,179; 930,254; 930,346; 930,450; 920,542; 850,588; 760,588; 680,577</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>仅作为导航记忆数据，常规地图不绘制</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>通路</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>central-spine</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>470,129; 470,208; 470,288; 470,369; 470,450; 470,531; 470,588</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>仅作为导航记忆数据，常规地图不绘制</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>通路</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>central-west</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>470,231; 420,231; 370,248; 330,277; 300,317; 300,369; 300,450; 340,496; 400,531; 470,531</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>仅作为导航记忆数据，常规地图不绘制</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>通路</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>central-east</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>470,242; 520,242; 570,254; 620,277; 660,323; 680,381; 650,450; 650,531; 650,588</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>仅作为导航记忆数据，常规地图不绘制</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>通路</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>sports-ring</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>680,150; 720,150; 800,150; 870,173; 910,231; 910,323; 910,415; 870,485; 800,508; 720,485; 680,450</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>仅作为导航记忆数据，常规地图不绘制</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>通路</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>south-cross</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>300,577; 380,577; 470,577; 560,577; 650,577; 720,588; 800,612; 900,612</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>仅作为导航记忆数据，常规地图不绘制</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>通路</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>lower-east</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>1</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>650,577; 650,635; 740,635; 830,635; 930,635</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>仅作为导航记忆数据，常规地图不绘制</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>通路</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>activity-center-2f</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>2</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>510,202; 550,190; 600,190; 650,208; 660,254; 635,294; 600,317; 555,312; 520,283; 510,237</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>仅作为导航记忆数据，常规地图不绘制</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>楼梯</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>only-purple-stair</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>1↔2</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>二层 635,294；一层 650,363</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>紫线垂直投影；唯一换层节点</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>障碍边界</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>campus-boundary</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>全部</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>15,87; 954,87; 973,114; 973,642; 933,685; 46,685; 15,87</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>不可通行；蓝色内部通路例外</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>障碍边界</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>sports-boundary</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>全部</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>760,138; 940,138; 940,635; 760,635; 760,138</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>不可通行；蓝色内部通路例外</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>障碍边界</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>indoor-gym-boundary</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>全部</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>690,121; 770,121; 770,219; 690,219; 690,121</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>不可通行；蓝色内部通路例外</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>障碍边界</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>activity-building-boundary</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>全部</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>500,173; 680,173; 680,335; 500,335; 500,173</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>不可通行；蓝色内部通路例外</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>障碍边界</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>teaching-building-boundary</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>全部</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>300,323; 620,323; 620,427; 300,427; 300,323</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>不可通行；蓝色内部通路例外</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>障碍边界</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>library-building-boundary</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>全部</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>300,444; 450,444; 450,577; 300,577; 300,444</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>不可通行；蓝色内部通路例外</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>障碍边界</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>dorm-service-boundary</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>全部</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>650,577; 930,577; 930,658; 650,658; 650,577</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>不可通行；蓝色内部通路例外</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:E18"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3245,56 +2917,68 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>底图像素</t>
+          <t>SVG坐标范围</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1448 × 1086</t>
+          <t>X 0–1000，Y 0–750</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SVG坐标范围</t>
+          <t>路网坐标</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>X 0–1000，Y 0–750</t>
+          <t>mapX / mapY，保持上一版路线连接</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>坐标版本</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>2</v>
+          <t>图标坐标</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>markerX / markerY，本次仅调整显示位置</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>内容版本</t>
+          <t>坐标版本</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>备注</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>圆点已按类实景底图建筑/入口中心重新校准；黑色斜杠区域 POI 保留在数据中但用户端隐藏。</t>
+          <t>内容版本</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>本次修改</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>仅复核 POI 图标坐标、缩小圆点、改为亮眼浅蓝标签；底图、路网和未探索区域路网范围不变。</t>
         </is>
       </c>
     </row>

</xml_diff>